<commit_message>
Backup: Save Firebase integration work before revert
</commit_message>
<xml_diff>
--- a/backend/Mandanten/Elektroniker_Testbetrieb/Angebote/angebote.xlsx
+++ b/backend/Mandanten/Elektroniker_Testbetrieb/Angebote/angebote.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -454,7 +454,7 @@
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="37" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -602,6 +602,43 @@
       <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Angebot_ANG-2026-001.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>ANG-2026-001</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Oma_Erna</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>435.00</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>517.65</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Angebot_ANG-2026-001_1767399233.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix protocol generation, list logic, and PDF download links
</commit_message>
<xml_diff>
--- a/backend/Mandanten/Elektroniker_Testbetrieb/Angebote/angebote.xlsx
+++ b/backend/Mandanten/Elektroniker_Testbetrieb/Angebote/angebote.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -454,7 +454,7 @@
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="37" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -602,6 +602,80 @@
       <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Angebot_ANG-2026-001.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>ANG-2026-001</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-04</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Oma_Erna</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>335.00</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>398.65</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Angebot_ANG-2026-001_1767556058.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>ANG-2026-001</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-04</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Oma_Erna</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>620.00</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>737.80</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Angebot_ANG-2026-001_1767560730.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>